<commit_message>
Add SQL scripts and README for Order Management Database System
</commit_message>
<xml_diff>
--- a/Excel/PR_2/PR2_Sales_Analytics.xlsx
+++ b/Excel/PR_2/PR2_Sales_Analytics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Priyansh\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Priyansh\OneDrive\Desktop\RW_Exam\Excel\PR_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27385E1C-D91C-47B2-83E5-2F702A450BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB7F7AB2-2E98-4300-AC5C-1C4D6E6C4C1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INDEX" sheetId="1" r:id="rId1"/>
@@ -1503,10 +1503,10 @@
     <xf numFmtId="170" fontId="2" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1516,10 +1516,6 @@
     <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1532,6 +1528,10 @@
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1541,19 +1541,58 @@
     <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1562,50 +1601,11 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3137,7 +3137,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr sz="1800" b="1" strike="noStrike" spc="-1">
+              <a:rPr lang="en-IN" sz="1800" b="1" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -3454,7 +3454,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr sz="1800" b="1" strike="noStrike" spc="-1">
+              <a:rPr lang="en-IN" sz="1800" b="1" strike="noStrike" spc="-1">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -4704,12 +4704,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="99" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
@@ -4902,20 +4902,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="100" t="s">
         <v>252</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
-      <c r="K1" s="99"/>
-      <c r="L1" s="99"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
+      <c r="H1" s="100"/>
+      <c r="I1" s="100"/>
+      <c r="J1" s="100"/>
+      <c r="K1" s="100"/>
+      <c r="L1" s="100"/>
     </row>
     <row r="3" spans="1:12" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -5141,264 +5141,280 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="113" t="s">
         <v>255</v>
       </c>
-      <c r="B1" s="132"/>
-      <c r="C1" s="132"/>
-      <c r="D1" s="132"/>
-      <c r="E1" s="132"/>
-      <c r="F1" s="132"/>
-      <c r="G1" s="132"/>
-      <c r="H1" s="132"/>
-      <c r="I1" s="132"/>
-      <c r="J1" s="132"/>
-      <c r="K1" s="132"/>
-      <c r="L1" s="132"/>
+      <c r="B1" s="113"/>
+      <c r="C1" s="113"/>
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
+      <c r="F1" s="113"/>
+      <c r="G1" s="113"/>
+      <c r="H1" s="113"/>
+      <c r="I1" s="113"/>
+      <c r="J1" s="113"/>
+      <c r="K1" s="113"/>
+      <c r="L1" s="113"/>
     </row>
     <row r="2" spans="1:12" ht="6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="132"/>
-      <c r="B2" s="132"/>
-      <c r="C2" s="132"/>
-      <c r="D2" s="132"/>
-      <c r="E2" s="132"/>
-      <c r="F2" s="132"/>
-      <c r="G2" s="132"/>
-      <c r="H2" s="132"/>
-      <c r="I2" s="132"/>
-      <c r="J2" s="132"/>
-      <c r="K2" s="132"/>
-      <c r="L2" s="132"/>
+      <c r="A2" s="113"/>
+      <c r="B2" s="113"/>
+      <c r="C2" s="113"/>
+      <c r="D2" s="113"/>
+      <c r="E2" s="113"/>
+      <c r="F2" s="113"/>
+      <c r="G2" s="113"/>
+      <c r="H2" s="113"/>
+      <c r="I2" s="113"/>
+      <c r="J2" s="113"/>
+      <c r="K2" s="113"/>
+      <c r="L2" s="113"/>
     </row>
     <row r="3" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="133" t="s">
+      <c r="A3" s="114" t="s">
         <v>256</v>
       </c>
-      <c r="B3" s="133"/>
-      <c r="C3" s="133"/>
-      <c r="D3" s="122" t="s">
+      <c r="B3" s="114"/>
+      <c r="C3" s="114"/>
+      <c r="D3" s="115" t="s">
         <v>257</v>
       </c>
-      <c r="E3" s="122"/>
-      <c r="F3" s="122"/>
-      <c r="G3" s="120" t="s">
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="116" t="s">
         <v>258</v>
       </c>
-      <c r="H3" s="120"/>
-      <c r="I3" s="120"/>
-      <c r="J3" s="134" t="s">
+      <c r="H3" s="116"/>
+      <c r="I3" s="116"/>
+      <c r="J3" s="117" t="s">
         <v>259</v>
       </c>
-      <c r="K3" s="134"/>
-      <c r="L3" s="134"/>
+      <c r="K3" s="117"/>
+      <c r="L3" s="117"/>
     </row>
     <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="128" t="s">
+      <c r="A4" s="118" t="s">
         <v>260</v>
       </c>
-      <c r="B4" s="128"/>
-      <c r="C4" s="128"/>
-      <c r="D4" s="126" t="s">
+      <c r="B4" s="118"/>
+      <c r="C4" s="118"/>
+      <c r="D4" s="119" t="s">
         <v>261</v>
       </c>
-      <c r="E4" s="126"/>
-      <c r="F4" s="126"/>
-      <c r="G4" s="124" t="s">
+      <c r="E4" s="119"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="120" t="s">
         <v>262</v>
       </c>
-      <c r="H4" s="124"/>
-      <c r="I4" s="124"/>
-      <c r="J4" s="129" t="s">
+      <c r="H4" s="120"/>
+      <c r="I4" s="120"/>
+      <c r="J4" s="121" t="s">
         <v>263</v>
       </c>
-      <c r="K4" s="129"/>
-      <c r="L4" s="129"/>
+      <c r="K4" s="121"/>
+      <c r="L4" s="121"/>
     </row>
     <row r="5" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="130" t="s">
+      <c r="A5" s="122" t="s">
         <v>264</v>
       </c>
-      <c r="B5" s="130"/>
-      <c r="C5" s="130"/>
-      <c r="D5" s="117" t="s">
+      <c r="B5" s="122"/>
+      <c r="C5" s="122"/>
+      <c r="D5" s="123" t="s">
         <v>265</v>
       </c>
-      <c r="E5" s="117"/>
-      <c r="F5" s="117"/>
-      <c r="G5" s="115" t="s">
+      <c r="E5" s="123"/>
+      <c r="F5" s="123"/>
+      <c r="G5" s="124" t="s">
         <v>266</v>
       </c>
-      <c r="H5" s="115"/>
-      <c r="I5" s="115"/>
-      <c r="J5" s="131" t="s">
+      <c r="H5" s="124"/>
+      <c r="I5" s="124"/>
+      <c r="J5" s="125" t="s">
         <v>267</v>
       </c>
-      <c r="K5" s="131"/>
-      <c r="L5" s="131"/>
+      <c r="K5" s="125"/>
+      <c r="L5" s="125"/>
     </row>
     <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="116" t="s">
         <v>268</v>
       </c>
-      <c r="B7" s="120"/>
-      <c r="C7" s="120"/>
-      <c r="D7" s="121" t="s">
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="126" t="s">
         <v>269</v>
       </c>
-      <c r="E7" s="121"/>
-      <c r="F7" s="121"/>
-      <c r="G7" s="122" t="s">
+      <c r="E7" s="126"/>
+      <c r="F7" s="126"/>
+      <c r="G7" s="115" t="s">
         <v>270</v>
       </c>
-      <c r="H7" s="122"/>
-      <c r="I7" s="122"/>
-      <c r="J7" s="123" t="s">
+      <c r="H7" s="115"/>
+      <c r="I7" s="115"/>
+      <c r="J7" s="127" t="s">
         <v>271</v>
       </c>
-      <c r="K7" s="123"/>
-      <c r="L7" s="123"/>
+      <c r="K7" s="127"/>
+      <c r="L7" s="127"/>
     </row>
     <row r="8" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="124" t="s">
+      <c r="A8" s="120" t="s">
         <v>105</v>
       </c>
-      <c r="B8" s="124"/>
-      <c r="C8" s="124"/>
-      <c r="D8" s="125" t="s">
+      <c r="B8" s="120"/>
+      <c r="C8" s="120"/>
+      <c r="D8" s="128" t="s">
         <v>59</v>
       </c>
-      <c r="E8" s="125"/>
-      <c r="F8" s="125"/>
-      <c r="G8" s="126" t="s">
+      <c r="E8" s="128"/>
+      <c r="F8" s="128"/>
+      <c r="G8" s="119" t="s">
         <v>58</v>
       </c>
-      <c r="H8" s="126"/>
-      <c r="I8" s="126"/>
-      <c r="J8" s="127" t="s">
+      <c r="H8" s="119"/>
+      <c r="I8" s="119"/>
+      <c r="J8" s="129" t="s">
         <v>272</v>
       </c>
-      <c r="K8" s="127"/>
-      <c r="L8" s="127"/>
+      <c r="K8" s="129"/>
+      <c r="L8" s="129"/>
     </row>
     <row r="9" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="115" t="s">
+      <c r="A9" s="124" t="s">
         <v>273</v>
       </c>
-      <c r="B9" s="115"/>
-      <c r="C9" s="115"/>
-      <c r="D9" s="116" t="s">
+      <c r="B9" s="124"/>
+      <c r="C9" s="124"/>
+      <c r="D9" s="130" t="s">
         <v>274</v>
       </c>
-      <c r="E9" s="116"/>
-      <c r="F9" s="116"/>
-      <c r="G9" s="117" t="s">
+      <c r="E9" s="130"/>
+      <c r="F9" s="130"/>
+      <c r="G9" s="123" t="s">
         <v>275</v>
       </c>
-      <c r="H9" s="117"/>
-      <c r="I9" s="117"/>
-      <c r="J9" s="118" t="s">
+      <c r="H9" s="123"/>
+      <c r="I9" s="123"/>
+      <c r="J9" s="131" t="s">
         <v>276</v>
       </c>
-      <c r="K9" s="118"/>
-      <c r="L9" s="118"/>
+      <c r="K9" s="131"/>
+      <c r="L9" s="131"/>
     </row>
     <row r="28" spans="7:12" x14ac:dyDescent="0.3">
-      <c r="G28" s="119" t="s">
+      <c r="G28" s="132" t="s">
         <v>277</v>
       </c>
-      <c r="H28" s="119"/>
-      <c r="I28" s="119"/>
-      <c r="J28" s="119"/>
-      <c r="K28" s="119"/>
-      <c r="L28" s="119"/>
+      <c r="H28" s="132"/>
+      <c r="I28" s="132"/>
+      <c r="J28" s="132"/>
+      <c r="K28" s="132"/>
+      <c r="L28" s="132"/>
     </row>
     <row r="29" spans="7:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G29" s="114" t="s">
+      <c r="G29" s="134" t="s">
         <v>278</v>
       </c>
-      <c r="H29" s="114"/>
-      <c r="I29" s="114"/>
-      <c r="J29" s="114"/>
-      <c r="K29" s="114"/>
-      <c r="L29" s="114"/>
+      <c r="H29" s="134"/>
+      <c r="I29" s="134"/>
+      <c r="J29" s="134"/>
+      <c r="K29" s="134"/>
+      <c r="L29" s="134"/>
     </row>
     <row r="30" spans="7:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G30" s="113" t="s">
+      <c r="G30" s="133" t="s">
         <v>279</v>
       </c>
-      <c r="H30" s="113"/>
-      <c r="I30" s="113"/>
-      <c r="J30" s="113"/>
-      <c r="K30" s="113"/>
-      <c r="L30" s="113"/>
+      <c r="H30" s="133"/>
+      <c r="I30" s="133"/>
+      <c r="J30" s="133"/>
+      <c r="K30" s="133"/>
+      <c r="L30" s="133"/>
     </row>
     <row r="31" spans="7:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G31" s="114" t="s">
+      <c r="G31" s="134" t="s">
         <v>280</v>
       </c>
-      <c r="H31" s="114"/>
-      <c r="I31" s="114"/>
-      <c r="J31" s="114"/>
-      <c r="K31" s="114"/>
-      <c r="L31" s="114"/>
+      <c r="H31" s="134"/>
+      <c r="I31" s="134"/>
+      <c r="J31" s="134"/>
+      <c r="K31" s="134"/>
+      <c r="L31" s="134"/>
     </row>
     <row r="32" spans="7:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G32" s="113" t="s">
+      <c r="G32" s="133" t="s">
         <v>281</v>
       </c>
-      <c r="H32" s="113"/>
-      <c r="I32" s="113"/>
-      <c r="J32" s="113"/>
-      <c r="K32" s="113"/>
-      <c r="L32" s="113"/>
+      <c r="H32" s="133"/>
+      <c r="I32" s="133"/>
+      <c r="J32" s="133"/>
+      <c r="K32" s="133"/>
+      <c r="L32" s="133"/>
     </row>
     <row r="33" spans="7:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G33" s="114" t="s">
+      <c r="G33" s="134" t="s">
         <v>282</v>
       </c>
-      <c r="H33" s="114"/>
-      <c r="I33" s="114"/>
-      <c r="J33" s="114"/>
-      <c r="K33" s="114"/>
-      <c r="L33" s="114"/>
+      <c r="H33" s="134"/>
+      <c r="I33" s="134"/>
+      <c r="J33" s="134"/>
+      <c r="K33" s="134"/>
+      <c r="L33" s="134"/>
     </row>
     <row r="34" spans="7:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G34" s="113" t="s">
+      <c r="G34" s="133" t="s">
         <v>283</v>
       </c>
-      <c r="H34" s="113"/>
-      <c r="I34" s="113"/>
-      <c r="J34" s="113"/>
-      <c r="K34" s="113"/>
-      <c r="L34" s="113"/>
+      <c r="H34" s="133"/>
+      <c r="I34" s="133"/>
+      <c r="J34" s="133"/>
+      <c r="K34" s="133"/>
+      <c r="L34" s="133"/>
     </row>
     <row r="35" spans="7:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G35" s="114" t="s">
+      <c r="G35" s="134" t="s">
         <v>284</v>
       </c>
-      <c r="H35" s="114"/>
-      <c r="I35" s="114"/>
-      <c r="J35" s="114"/>
-      <c r="K35" s="114"/>
-      <c r="L35" s="114"/>
+      <c r="H35" s="134"/>
+      <c r="I35" s="134"/>
+      <c r="J35" s="134"/>
+      <c r="K35" s="134"/>
+      <c r="L35" s="134"/>
     </row>
     <row r="36" spans="7:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G36" s="113" t="s">
+      <c r="G36" s="133" t="s">
         <v>285</v>
       </c>
-      <c r="H36" s="113"/>
-      <c r="I36" s="113"/>
-      <c r="J36" s="113"/>
-      <c r="K36" s="113"/>
-      <c r="L36" s="113"/>
+      <c r="H36" s="133"/>
+      <c r="I36" s="133"/>
+      <c r="J36" s="133"/>
+      <c r="K36" s="133"/>
+      <c r="L36" s="133"/>
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="A1:L2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="J3:L3"/>
+    <mergeCell ref="G34:L34"/>
+    <mergeCell ref="G35:L35"/>
+    <mergeCell ref="G36:L36"/>
+    <mergeCell ref="G29:L29"/>
+    <mergeCell ref="G30:L30"/>
+    <mergeCell ref="G31:L31"/>
+    <mergeCell ref="G32:L32"/>
+    <mergeCell ref="G33:L33"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="G28:L28"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="J8:L8"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="G4:I4"/>
@@ -5407,27 +5423,11 @@
     <mergeCell ref="D5:F5"/>
     <mergeCell ref="G5:I5"/>
     <mergeCell ref="J5:L5"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="J8:L8"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="G28:L28"/>
-    <mergeCell ref="G34:L34"/>
-    <mergeCell ref="G35:L35"/>
-    <mergeCell ref="G36:L36"/>
-    <mergeCell ref="G29:L29"/>
-    <mergeCell ref="G30:L30"/>
-    <mergeCell ref="G31:L31"/>
-    <mergeCell ref="G32:L32"/>
-    <mergeCell ref="G33:L33"/>
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="J3:L3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5514,7 +5514,7 @@
       </c>
       <c r="J2" s="13">
         <f t="shared" ref="J2:J33" ca="1" si="0">NOW()</f>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -5547,7 +5547,7 @@
       </c>
       <c r="J3" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -5580,7 +5580,7 @@
       </c>
       <c r="J4" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -5613,7 +5613,7 @@
       </c>
       <c r="J5" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -5646,7 +5646,7 @@
       </c>
       <c r="J6" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -5679,7 +5679,7 @@
       </c>
       <c r="J7" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J8" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="J9" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
@@ -5778,7 +5778,7 @@
       </c>
       <c r="J10" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -5811,7 +5811,7 @@
       </c>
       <c r="J11" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
@@ -5844,7 +5844,7 @@
       </c>
       <c r="J12" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
@@ -5877,7 +5877,7 @@
       </c>
       <c r="J13" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
@@ -5910,7 +5910,7 @@
       </c>
       <c r="J14" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
@@ -5943,7 +5943,7 @@
       </c>
       <c r="J15" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
@@ -5976,7 +5976,7 @@
       </c>
       <c r="J16" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
@@ -6009,7 +6009,7 @@
       </c>
       <c r="J17" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
@@ -6042,7 +6042,7 @@
       </c>
       <c r="J18" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
@@ -6075,7 +6075,7 @@
       </c>
       <c r="J19" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
@@ -6108,7 +6108,7 @@
       </c>
       <c r="J20" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
@@ -6141,7 +6141,7 @@
       </c>
       <c r="J21" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
@@ -6174,7 +6174,7 @@
       </c>
       <c r="J22" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="J23" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="J24" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
@@ -6273,7 +6273,7 @@
       </c>
       <c r="J25" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="J26" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="J27" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
@@ -6372,7 +6372,7 @@
       </c>
       <c r="J28" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="J29" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
@@ -6438,7 +6438,7 @@
       </c>
       <c r="J30" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
@@ -6471,7 +6471,7 @@
       </c>
       <c r="J31" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
@@ -6504,7 +6504,7 @@
       </c>
       <c r="J32" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
@@ -6537,7 +6537,7 @@
       </c>
       <c r="J33" s="13">
         <f t="shared" ca="1" si="0"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
@@ -6570,7 +6570,7 @@
       </c>
       <c r="J34" s="13">
         <f t="shared" ref="J34:J65" ca="1" si="1">NOW()</f>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="J35" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
@@ -6636,7 +6636,7 @@
       </c>
       <c r="J36" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
@@ -6669,7 +6669,7 @@
       </c>
       <c r="J37" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
@@ -6702,7 +6702,7 @@
       </c>
       <c r="J38" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="J39" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
@@ -6768,7 +6768,7 @@
       </c>
       <c r="J40" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
@@ -6801,7 +6801,7 @@
       </c>
       <c r="J41" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
@@ -6834,7 +6834,7 @@
       </c>
       <c r="J42" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
@@ -6867,7 +6867,7 @@
       </c>
       <c r="J43" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
@@ -6900,7 +6900,7 @@
       </c>
       <c r="J44" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="J45" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
@@ -6966,7 +6966,7 @@
       </c>
       <c r="J46" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
@@ -6999,7 +6999,7 @@
       </c>
       <c r="J47" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
@@ -7032,7 +7032,7 @@
       </c>
       <c r="J48" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
@@ -7065,7 +7065,7 @@
       </c>
       <c r="J49" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
@@ -7098,7 +7098,7 @@
       </c>
       <c r="J50" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="J51" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="J52" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
@@ -7197,7 +7197,7 @@
       </c>
       <c r="J53" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
@@ -7230,7 +7230,7 @@
       </c>
       <c r="J54" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="J55" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
@@ -7296,7 +7296,7 @@
       </c>
       <c r="J56" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
@@ -7329,7 +7329,7 @@
       </c>
       <c r="J57" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
@@ -7362,7 +7362,7 @@
       </c>
       <c r="J58" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="J59" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
@@ -7428,7 +7428,7 @@
       </c>
       <c r="J60" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
@@ -7461,7 +7461,7 @@
       </c>
       <c r="J61" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="J62" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
@@ -7527,7 +7527,7 @@
       </c>
       <c r="J63" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
@@ -7560,7 +7560,7 @@
       </c>
       <c r="J64" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
@@ -7593,7 +7593,7 @@
       </c>
       <c r="J65" s="13">
         <f t="shared" ca="1" si="1"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
@@ -7626,7 +7626,7 @@
       </c>
       <c r="J66" s="13">
         <f t="shared" ref="J66:J97" ca="1" si="2">NOW()</f>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="J67" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="J68" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
@@ -7725,7 +7725,7 @@
       </c>
       <c r="J69" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="J70" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
@@ -7791,7 +7791,7 @@
       </c>
       <c r="J71" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J72" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
@@ -7857,7 +7857,7 @@
       </c>
       <c r="J73" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
@@ -7890,7 +7890,7 @@
       </c>
       <c r="J74" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.3">
@@ -7923,7 +7923,7 @@
       </c>
       <c r="J75" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
@@ -7956,7 +7956,7 @@
       </c>
       <c r="J76" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="J77" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
@@ -8022,7 +8022,7 @@
       </c>
       <c r="J78" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.3">
@@ -8055,7 +8055,7 @@
       </c>
       <c r="J79" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.3">
@@ -8088,7 +8088,7 @@
       </c>
       <c r="J80" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.3">
@@ -8121,7 +8121,7 @@
       </c>
       <c r="J81" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.3">
@@ -8154,7 +8154,7 @@
       </c>
       <c r="J82" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.3">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="J83" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.3">
@@ -8220,7 +8220,7 @@
       </c>
       <c r="J84" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.3">
@@ -8253,7 +8253,7 @@
       </c>
       <c r="J85" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.3">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="J86" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.3">
@@ -8319,7 +8319,7 @@
       </c>
       <c r="J87" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.3">
@@ -8352,7 +8352,7 @@
       </c>
       <c r="J88" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.3">
@@ -8385,7 +8385,7 @@
       </c>
       <c r="J89" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.3">
@@ -8418,7 +8418,7 @@
       </c>
       <c r="J90" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.3">
@@ -8451,7 +8451,7 @@
       </c>
       <c r="J91" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.3">
@@ -8484,7 +8484,7 @@
       </c>
       <c r="J92" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.3">
@@ -8517,7 +8517,7 @@
       </c>
       <c r="J93" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.3">
@@ -8550,7 +8550,7 @@
       </c>
       <c r="J94" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.3">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="J95" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.3">
@@ -8616,7 +8616,7 @@
       </c>
       <c r="J96" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.3">
@@ -8649,7 +8649,7 @@
       </c>
       <c r="J97" s="13">
         <f t="shared" ca="1" si="2"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.3">
@@ -8682,7 +8682,7 @@
       </c>
       <c r="J98" s="13">
         <f t="shared" ref="J98:J129" ca="1" si="3">NOW()</f>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.3">
@@ -8715,7 +8715,7 @@
       </c>
       <c r="J99" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.3">
@@ -8748,7 +8748,7 @@
       </c>
       <c r="J100" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.3">
@@ -8781,7 +8781,7 @@
       </c>
       <c r="J101" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.3">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="J102" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.3">
@@ -8847,7 +8847,7 @@
       </c>
       <c r="J103" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.3">
@@ -8880,7 +8880,7 @@
       </c>
       <c r="J104" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.3">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="J105" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.3">
@@ -8946,7 +8946,7 @@
       </c>
       <c r="J106" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.3">
@@ -8979,7 +8979,7 @@
       </c>
       <c r="J107" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.3">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="J108" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.3">
@@ -9045,7 +9045,7 @@
       </c>
       <c r="J109" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.3">
@@ -9078,7 +9078,7 @@
       </c>
       <c r="J110" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.3">
@@ -9111,7 +9111,7 @@
       </c>
       <c r="J111" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.3">
@@ -9144,7 +9144,7 @@
       </c>
       <c r="J112" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.3">
@@ -9177,7 +9177,7 @@
       </c>
       <c r="J113" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.3">
@@ -9210,7 +9210,7 @@
       </c>
       <c r="J114" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.3">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="J115" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.3">
@@ -9276,7 +9276,7 @@
       </c>
       <c r="J116" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.3">
@@ -9309,7 +9309,7 @@
       </c>
       <c r="J117" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.3">
@@ -9342,7 +9342,7 @@
       </c>
       <c r="J118" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.3">
@@ -9375,7 +9375,7 @@
       </c>
       <c r="J119" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.3">
@@ -9408,7 +9408,7 @@
       </c>
       <c r="J120" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.3">
@@ -9441,7 +9441,7 @@
       </c>
       <c r="J121" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.3">
@@ -9474,7 +9474,7 @@
       </c>
       <c r="J122" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.3">
@@ -9507,7 +9507,7 @@
       </c>
       <c r="J123" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.3">
@@ -9540,7 +9540,7 @@
       </c>
       <c r="J124" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.3">
@@ -9573,7 +9573,7 @@
       </c>
       <c r="J125" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.3">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="J126" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="127" spans="1:10" x14ac:dyDescent="0.3">
@@ -9639,7 +9639,7 @@
       </c>
       <c r="J127" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="128" spans="1:10" x14ac:dyDescent="0.3">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="J128" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.3">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="J129" s="13">
         <f t="shared" ca="1" si="3"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.3">
@@ -9738,7 +9738,7 @@
       </c>
       <c r="J130" s="13">
         <f t="shared" ref="J130:J161" ca="1" si="4">NOW()</f>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.3">
@@ -9771,7 +9771,7 @@
       </c>
       <c r="J131" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.3">
@@ -9804,7 +9804,7 @@
       </c>
       <c r="J132" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.3">
@@ -9837,7 +9837,7 @@
       </c>
       <c r="J133" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.3">
@@ -9870,7 +9870,7 @@
       </c>
       <c r="J134" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.3">
@@ -9903,7 +9903,7 @@
       </c>
       <c r="J135" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.3">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="J136" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.3">
@@ -9969,7 +9969,7 @@
       </c>
       <c r="J137" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.3">
@@ -10002,7 +10002,7 @@
       </c>
       <c r="J138" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.3">
@@ -10035,7 +10035,7 @@
       </c>
       <c r="J139" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.3">
@@ -10068,7 +10068,7 @@
       </c>
       <c r="J140" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.3">
@@ -10101,7 +10101,7 @@
       </c>
       <c r="J141" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.3">
@@ -10134,7 +10134,7 @@
       </c>
       <c r="J142" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.3">
@@ -10167,7 +10167,7 @@
       </c>
       <c r="J143" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.3">
@@ -10200,7 +10200,7 @@
       </c>
       <c r="J144" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.3">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="J145" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.3">
@@ -10266,7 +10266,7 @@
       </c>
       <c r="J146" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="147" spans="1:10" x14ac:dyDescent="0.3">
@@ -10299,7 +10299,7 @@
       </c>
       <c r="J147" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="148" spans="1:10" x14ac:dyDescent="0.3">
@@ -10332,7 +10332,7 @@
       </c>
       <c r="J148" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="149" spans="1:10" x14ac:dyDescent="0.3">
@@ -10365,7 +10365,7 @@
       </c>
       <c r="J149" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="150" spans="1:10" x14ac:dyDescent="0.3">
@@ -10398,7 +10398,7 @@
       </c>
       <c r="J150" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.3">
@@ -10431,7 +10431,7 @@
       </c>
       <c r="J151" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="152" spans="1:10" x14ac:dyDescent="0.3">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="J152" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.3">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="J153" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="154" spans="1:10" x14ac:dyDescent="0.3">
@@ -10530,7 +10530,7 @@
       </c>
       <c r="J154" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="155" spans="1:10" x14ac:dyDescent="0.3">
@@ -10563,7 +10563,7 @@
       </c>
       <c r="J155" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="156" spans="1:10" x14ac:dyDescent="0.3">
@@ -10596,7 +10596,7 @@
       </c>
       <c r="J156" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="157" spans="1:10" x14ac:dyDescent="0.3">
@@ -10629,7 +10629,7 @@
       </c>
       <c r="J157" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.3">
@@ -10662,7 +10662,7 @@
       </c>
       <c r="J158" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="159" spans="1:10" x14ac:dyDescent="0.3">
@@ -10695,7 +10695,7 @@
       </c>
       <c r="J159" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.3">
@@ -10728,7 +10728,7 @@
       </c>
       <c r="J160" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="161" spans="1:10" x14ac:dyDescent="0.3">
@@ -10761,7 +10761,7 @@
       </c>
       <c r="J161" s="13">
         <f t="shared" ca="1" si="4"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.3">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="J162" s="13">
         <f t="shared" ref="J162:J193" ca="1" si="5">NOW()</f>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.3">
@@ -10827,7 +10827,7 @@
       </c>
       <c r="J163" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.3">
@@ -10860,7 +10860,7 @@
       </c>
       <c r="J164" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.3">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="J165" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="166" spans="1:10" x14ac:dyDescent="0.3">
@@ -10926,7 +10926,7 @@
       </c>
       <c r="J166" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.3">
@@ -10959,7 +10959,7 @@
       </c>
       <c r="J167" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.3">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="J168" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="169" spans="1:10" x14ac:dyDescent="0.3">
@@ -11025,7 +11025,7 @@
       </c>
       <c r="J169" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.3">
@@ -11058,7 +11058,7 @@
       </c>
       <c r="J170" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.3">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="J171" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.3">
@@ -11124,7 +11124,7 @@
       </c>
       <c r="J172" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="173" spans="1:10" x14ac:dyDescent="0.3">
@@ -11157,7 +11157,7 @@
       </c>
       <c r="J173" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.3">
@@ -11190,7 +11190,7 @@
       </c>
       <c r="J174" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="175" spans="1:10" x14ac:dyDescent="0.3">
@@ -11223,7 +11223,7 @@
       </c>
       <c r="J175" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="176" spans="1:10" x14ac:dyDescent="0.3">
@@ -11256,7 +11256,7 @@
       </c>
       <c r="J176" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="177" spans="1:10" x14ac:dyDescent="0.3">
@@ -11289,7 +11289,7 @@
       </c>
       <c r="J177" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="178" spans="1:10" x14ac:dyDescent="0.3">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="J178" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="179" spans="1:10" x14ac:dyDescent="0.3">
@@ -11355,7 +11355,7 @@
       </c>
       <c r="J179" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="180" spans="1:10" x14ac:dyDescent="0.3">
@@ -11388,7 +11388,7 @@
       </c>
       <c r="J180" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="181" spans="1:10" x14ac:dyDescent="0.3">
@@ -11421,7 +11421,7 @@
       </c>
       <c r="J181" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="182" spans="1:10" x14ac:dyDescent="0.3">
@@ -11454,7 +11454,7 @@
       </c>
       <c r="J182" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="183" spans="1:10" x14ac:dyDescent="0.3">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="J183" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="184" spans="1:10" x14ac:dyDescent="0.3">
@@ -11520,7 +11520,7 @@
       </c>
       <c r="J184" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="185" spans="1:10" x14ac:dyDescent="0.3">
@@ -11553,7 +11553,7 @@
       </c>
       <c r="J185" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="186" spans="1:10" x14ac:dyDescent="0.3">
@@ -11586,7 +11586,7 @@
       </c>
       <c r="J186" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="187" spans="1:10" x14ac:dyDescent="0.3">
@@ -11619,7 +11619,7 @@
       </c>
       <c r="J187" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="188" spans="1:10" x14ac:dyDescent="0.3">
@@ -11652,7 +11652,7 @@
       </c>
       <c r="J188" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="189" spans="1:10" x14ac:dyDescent="0.3">
@@ -11685,7 +11685,7 @@
       </c>
       <c r="J189" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="190" spans="1:10" x14ac:dyDescent="0.3">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="J190" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="191" spans="1:10" x14ac:dyDescent="0.3">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="J191" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="192" spans="1:10" x14ac:dyDescent="0.3">
@@ -11784,7 +11784,7 @@
       </c>
       <c r="J192" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="193" spans="1:10" x14ac:dyDescent="0.3">
@@ -11817,7 +11817,7 @@
       </c>
       <c r="J193" s="13">
         <f t="shared" ca="1" si="5"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="194" spans="1:10" x14ac:dyDescent="0.3">
@@ -11850,7 +11850,7 @@
       </c>
       <c r="J194" s="13">
         <f t="shared" ref="J194:J201" ca="1" si="6">NOW()</f>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="195" spans="1:10" x14ac:dyDescent="0.3">
@@ -11883,7 +11883,7 @@
       </c>
       <c r="J195" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="196" spans="1:10" x14ac:dyDescent="0.3">
@@ -11916,7 +11916,7 @@
       </c>
       <c r="J196" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="197" spans="1:10" x14ac:dyDescent="0.3">
@@ -11949,7 +11949,7 @@
       </c>
       <c r="J197" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="198" spans="1:10" x14ac:dyDescent="0.3">
@@ -11982,7 +11982,7 @@
       </c>
       <c r="J198" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="199" spans="1:10" x14ac:dyDescent="0.3">
@@ -12015,7 +12015,7 @@
       </c>
       <c r="J199" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="200" spans="1:10" x14ac:dyDescent="0.3">
@@ -12048,7 +12048,7 @@
       </c>
       <c r="J200" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
     <row r="201" spans="1:10" x14ac:dyDescent="0.3">
@@ -12081,7 +12081,7 @@
       </c>
       <c r="J201" s="13">
         <f t="shared" ca="1" si="6"/>
-        <v>46108.653701620373</v>
+        <v>46108.667233912034</v>
       </c>
     </row>
   </sheetData>
@@ -12127,14 +12127,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="100" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
     </row>
     <row r="2" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -12400,15 +12400,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="100" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
     </row>
     <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="102" t="s">
@@ -12683,13 +12683,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="100" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="102" t="s">
@@ -13043,33 +13043,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="100" t="s">
         <v>184</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="106" t="s">
+      <c r="A2" s="104" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="106"/>
-      <c r="C2" s="107" t="s">
+      <c r="B2" s="104"/>
+      <c r="C2" s="105" t="s">
         <v>55</v>
       </c>
-      <c r="D2" s="107"/>
-      <c r="E2" s="108" t="s">
+      <c r="D2" s="105"/>
+      <c r="E2" s="106" t="s">
         <v>52</v>
       </c>
-      <c r="F2" s="108"/>
-      <c r="G2" s="109" t="s">
+      <c r="F2" s="106"/>
+      <c r="G2" s="107" t="s">
         <v>53</v>
       </c>
-      <c r="H2" s="109"/>
+      <c r="H2" s="107"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="63" t="s">
@@ -13488,77 +13488,77 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="104" t="s">
+      <c r="A20" s="108" t="s">
         <v>202</v>
       </c>
-      <c r="B20" s="104"/>
-      <c r="C20" s="104"/>
-      <c r="D20" s="104"/>
-      <c r="E20" s="104"/>
-      <c r="F20" s="104"/>
-      <c r="G20" s="104"/>
-      <c r="H20" s="104"/>
+      <c r="B20" s="108"/>
+      <c r="C20" s="108"/>
+      <c r="D20" s="108"/>
+      <c r="E20" s="108"/>
+      <c r="F20" s="108"/>
+      <c r="G20" s="108"/>
+      <c r="H20" s="108"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="105" t="s">
+      <c r="A21" s="109" t="s">
         <v>203</v>
       </c>
-      <c r="B21" s="105"/>
-      <c r="C21" s="105"/>
-      <c r="D21" s="105"/>
-      <c r="E21" s="105"/>
-      <c r="F21" s="105"/>
-      <c r="G21" s="105"/>
-      <c r="H21" s="105"/>
+      <c r="B21" s="109"/>
+      <c r="C21" s="109"/>
+      <c r="D21" s="109"/>
+      <c r="E21" s="109"/>
+      <c r="F21" s="109"/>
+      <c r="G21" s="109"/>
+      <c r="H21" s="109"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="105" t="s">
+      <c r="A22" s="109" t="s">
         <v>204</v>
       </c>
-      <c r="B22" s="105"/>
-      <c r="C22" s="105"/>
-      <c r="D22" s="105"/>
-      <c r="E22" s="105"/>
-      <c r="F22" s="105"/>
-      <c r="G22" s="105"/>
-      <c r="H22" s="105"/>
+      <c r="B22" s="109"/>
+      <c r="C22" s="109"/>
+      <c r="D22" s="109"/>
+      <c r="E22" s="109"/>
+      <c r="F22" s="109"/>
+      <c r="G22" s="109"/>
+      <c r="H22" s="109"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23" s="105" t="s">
+      <c r="A23" s="109" t="s">
         <v>205</v>
       </c>
-      <c r="B23" s="105"/>
-      <c r="C23" s="105"/>
-      <c r="D23" s="105"/>
-      <c r="E23" s="105"/>
-      <c r="F23" s="105"/>
-      <c r="G23" s="105"/>
-      <c r="H23" s="105"/>
+      <c r="B23" s="109"/>
+      <c r="C23" s="109"/>
+      <c r="D23" s="109"/>
+      <c r="E23" s="109"/>
+      <c r="F23" s="109"/>
+      <c r="G23" s="109"/>
+      <c r="H23" s="109"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="105" t="s">
+      <c r="A24" s="109" t="s">
         <v>206</v>
       </c>
-      <c r="B24" s="105"/>
-      <c r="C24" s="105"/>
-      <c r="D24" s="105"/>
-      <c r="E24" s="105"/>
-      <c r="F24" s="105"/>
-      <c r="G24" s="105"/>
-      <c r="H24" s="105"/>
+      <c r="B24" s="109"/>
+      <c r="C24" s="109"/>
+      <c r="D24" s="109"/>
+      <c r="E24" s="109"/>
+      <c r="F24" s="109"/>
+      <c r="G24" s="109"/>
+      <c r="H24" s="109"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A24:H24"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="G2:H2"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A24:H24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -13577,14 +13577,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="100" t="s">
         <v>207</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
     </row>
     <row r="2" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -13901,16 +13901,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="100" t="s">
         <v>232</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
+      <c r="H1" s="100"/>
     </row>
     <row r="2" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -14805,16 +14805,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="100" t="s">
         <v>248</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
+      <c r="H1" s="100"/>
     </row>
     <row r="2" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">

</xml_diff>